<commit_message>
Added the form for the data and the storing of data in json format
</commit_message>
<xml_diff>
--- a/Docs/Conza finale 0.xlsx
+++ b/Docs/Conza finale 0.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paolopalmiero/Documents/Lavoro/Invasi/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paolopalmiero/Documents/Lavoro/Invasi/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C243AE-CED3-4A49-A859-43BAA26CCF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37D2965-53BE-384E-B55F-5C7C9F27254E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7852,7 +7852,7 @@
         <v>18</v>
       </c>
       <c r="D10">
-        <f t="shared" ref="D10:D21" si="0">T10</f>
+        <f>T10</f>
         <v>2.4862538847716956E-2</v>
       </c>
       <c r="E10">
@@ -7893,7 +7893,7 @@
         <v>2.08</v>
       </c>
       <c r="T10">
-        <f t="shared" ref="T10:T21" si="1">R10/$S$21</f>
+        <f t="shared" ref="T10:T21" si="0">R10/$S$21</f>
         <v>2.4862538847716956E-2</v>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
         <v>20</v>
       </c>
       <c r="D11">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D10:D21" si="1">T11</f>
         <v>9.3951709299545799E-2</v>
       </c>
       <c r="E11">
@@ -7943,7 +7943,7 @@
         <v>9.9400000000000013</v>
       </c>
       <c r="T11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>9.3951709299545799E-2</v>
       </c>
     </row>
@@ -7952,7 +7952,7 @@
         <v>23</v>
       </c>
       <c r="D12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.15479321061439161</v>
       </c>
       <c r="E12">
@@ -7993,7 +7993,7 @@
         <v>22.89</v>
       </c>
       <c r="T12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.15479321061439161</v>
       </c>
     </row>
@@ -8002,7 +8002,7 @@
         <v>25</v>
       </c>
       <c r="D13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1711690174515898</v>
       </c>
       <c r="E13">
@@ -8043,7 +8043,7 @@
         <v>37.21</v>
       </c>
       <c r="T13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.1711690174515898</v>
       </c>
     </row>
@@ -8052,7 +8052,7 @@
         <v>27</v>
       </c>
       <c r="D14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.16925651446330389</v>
       </c>
       <c r="E14">
@@ -8093,7 +8093,7 @@
         <v>51.370000000000005</v>
       </c>
       <c r="T14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.16925651446330389</v>
       </c>
     </row>
@@ -8102,7 +8102,7 @@
         <v>29</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.18312216112837681</v>
       </c>
       <c r="E15">
@@ -8143,7 +8143,7 @@
         <v>66.69</v>
       </c>
       <c r="T15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.18312216112837681</v>
       </c>
     </row>
@@ -8152,7 +8152,7 @@
         <v>31</v>
       </c>
       <c r="D16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8.1879034185990934E-2</v>
       </c>
       <c r="E16">
@@ -8187,7 +8187,7 @@
         <v>73.539999999999992</v>
       </c>
       <c r="T16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>8.1879034185990934E-2</v>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
         <v>33</v>
       </c>
       <c r="D17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4.6617260339469287E-2</v>
       </c>
       <c r="E17">
@@ -8230,7 +8230,7 @@
         <v>77.44</v>
       </c>
       <c r="T17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4.6617260339469287E-2</v>
       </c>
     </row>
@@ -8239,7 +8239,7 @@
         <v>35</v>
       </c>
       <c r="D18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.7611761893377964E-2</v>
       </c>
       <c r="E18">
@@ -8273,7 +8273,7 @@
         <v>79.75</v>
       </c>
       <c r="T18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.7611761893377964E-2</v>
       </c>
     </row>
@@ -8282,7 +8282,7 @@
         <v>36</v>
       </c>
       <c r="D19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.7451589768109017E-2</v>
       </c>
       <c r="E19">
@@ -8316,7 +8316,7 @@
         <v>81.209999999999994</v>
       </c>
       <c r="T19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.7451589768109017E-2</v>
       </c>
     </row>
@@ -8325,7 +8325,7 @@
         <v>37</v>
       </c>
       <c r="D20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.3148458044465699E-2</v>
       </c>
       <c r="E20">
@@ -8359,7 +8359,7 @@
         <v>82.309999999999988</v>
       </c>
       <c r="T20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.3148458044465699E-2</v>
       </c>
     </row>
@@ -8368,7 +8368,7 @@
         <v>38</v>
       </c>
       <c r="D21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.6136743963662447E-2</v>
       </c>
       <c r="E21">
@@ -8402,7 +8402,7 @@
         <v>83.659999999999982</v>
       </c>
       <c r="T21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.6136743963662447E-2</v>
       </c>
     </row>
@@ -8884,7 +8884,7 @@
         <v>20</v>
       </c>
       <c r="D30">
-        <f t="shared" ref="D29:D40" si="10">D11*$O$10</f>
+        <f t="shared" ref="D30:D40" si="10">D11*$O$10</f>
         <v>7.8600000000000012</v>
       </c>
       <c r="E30">
@@ -8907,7 +8907,7 @@
         <v>9.9400000000000013</v>
       </c>
       <c r="J30">
-        <f t="shared" ref="J29:J40" si="12">H11*$O$12</f>
+        <f t="shared" ref="J30:J40" si="12">H11*$O$12</f>
         <v>0</v>
       </c>
       <c r="K30">
@@ -8915,7 +8915,7 @@
         <v>0</v>
       </c>
       <c r="L30">
-        <f t="shared" ref="L29:L40" si="13">I11*$O$13</f>
+        <f t="shared" ref="L30:L40" si="13">I11*$O$13</f>
         <v>2.5</v>
       </c>
       <c r="M30">
@@ -8923,7 +8923,7 @@
         <v>5</v>
       </c>
       <c r="N30">
-        <f t="shared" ref="N29:N40" si="14">J11*$O$14</f>
+        <f t="shared" ref="N30:N40" si="14">J11*$O$14</f>
         <v>0</v>
       </c>
       <c r="O30">
@@ -8931,7 +8931,7 @@
         <v>0</v>
       </c>
       <c r="P30">
-        <f t="shared" ref="P29:P40" si="15">K11*$O$15</f>
+        <f t="shared" ref="P30:P40" si="15">K11*$O$15</f>
         <v>0</v>
       </c>
       <c r="Q30">
@@ -8949,7 +8949,7 @@
         <v>0</v>
       </c>
       <c r="U30">
-        <f t="shared" ref="U29:U40" si="17">(J30+L30+N30+P30+R30)</f>
+        <f t="shared" ref="U30:U40" si="17">(J30+L30+N30+P30+R30)</f>
         <v>2.5</v>
       </c>
       <c r="V30" s="1">
@@ -8957,7 +8957,7 @@
         <v>5</v>
       </c>
       <c r="W30">
-        <f t="shared" ref="W29:W40" si="18">H30-U30</f>
+        <f t="shared" ref="W30:W40" si="18">H30-U30</f>
         <v>5.3600000000000012</v>
       </c>
       <c r="X30">

</xml_diff>

<commit_message>
Added the cumulative sums of data
</commit_message>
<xml_diff>
--- a/Docs/Conza finale 0.xlsx
+++ b/Docs/Conza finale 0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paolopalmiero/Documents/Lavoro/Invasi/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37D2965-53BE-384E-B55F-5C7C9F27254E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A35AC5-D5AF-BF41-AAAA-098C662E9B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7902,7 +7902,7 @@
         <v>20</v>
       </c>
       <c r="D11">
-        <f t="shared" ref="D10:D21" si="1">T11</f>
+        <f t="shared" ref="D11:D21" si="1">T11</f>
         <v>9.3951709299545799E-2</v>
       </c>
       <c r="E11">

</xml_diff>

<commit_message>
Added the generation of plots
</commit_message>
<xml_diff>
--- a/Docs/Conza finale 0.xlsx
+++ b/Docs/Conza finale 0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paolopalmiero/Documents/Lavoro/Invasi/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A35AC5-D5AF-BF41-AAAA-098C662E9B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BCC7A4-3D14-6445-84AA-802912A3D129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28800" yWindow="500" windowWidth="23600" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -8052,7 +8052,7 @@
         <v>27</v>
       </c>
       <c r="D14">
-        <f t="shared" si="1"/>
+        <f>T14</f>
         <v>0.16925651446330389</v>
       </c>
       <c r="E14">
@@ -8239,7 +8239,7 @@
         <v>35</v>
       </c>
       <c r="D18">
-        <f t="shared" si="1"/>
+        <f>T18</f>
         <v>2.7611761893377964E-2</v>
       </c>
       <c r="E18">
@@ -8368,7 +8368,7 @@
         <v>38</v>
       </c>
       <c r="D21">
-        <f t="shared" si="1"/>
+        <f>T21</f>
         <v>1.6136743963662447E-2</v>
       </c>
       <c r="E21">
@@ -10505,7 +10505,7 @@
         <v>2.5</v>
       </c>
       <c r="G46">
-        <f t="shared" ref="G46:G57" si="36">Z29</f>
+        <f>Z29</f>
         <v>18.080000000000002</v>
       </c>
       <c r="H46">
@@ -10530,15 +10530,15 @@
         <v>20</v>
       </c>
       <c r="E47">
-        <f t="shared" ref="E47:E57" si="37">I30</f>
+        <f t="shared" ref="E47:E57" si="36">I30</f>
         <v>9.9400000000000013</v>
       </c>
       <c r="F47">
-        <f t="shared" ref="F47:F57" si="38" xml:space="preserve"> V30</f>
+        <f t="shared" ref="F47:F57" si="37" xml:space="preserve"> V30</f>
         <v>5</v>
       </c>
       <c r="G47">
-        <f t="shared" si="36"/>
+        <f t="shared" ref="G46:G57" si="38">Z30</f>
         <v>23.44</v>
       </c>
       <c r="H47">
@@ -10563,15 +10563,15 @@
         <v>23</v>
       </c>
       <c r="E48">
+        <f t="shared" si="36"/>
+        <v>22.89</v>
+      </c>
+      <c r="F48">
         <f t="shared" si="37"/>
-        <v>22.89</v>
-      </c>
-      <c r="F48">
+        <v>7.5</v>
+      </c>
+      <c r="G48">
         <f t="shared" si="38"/>
-        <v>7.5</v>
-      </c>
-      <c r="G48">
-        <f t="shared" si="36"/>
         <v>33.89</v>
       </c>
       <c r="H48">
@@ -10596,15 +10596,15 @@
         <v>25</v>
       </c>
       <c r="E49">
+        <f t="shared" si="36"/>
+        <v>37.21</v>
+      </c>
+      <c r="F49">
         <f t="shared" si="37"/>
-        <v>37.21</v>
-      </c>
-      <c r="F49">
+        <v>10</v>
+      </c>
+      <c r="G49">
         <f t="shared" si="38"/>
-        <v>10</v>
-      </c>
-      <c r="G49">
-        <f t="shared" si="36"/>
         <v>45.710000000000008</v>
       </c>
       <c r="H49">
@@ -10638,15 +10638,15 @@
         <v>27</v>
       </c>
       <c r="E50">
+        <f t="shared" si="36"/>
+        <v>51.370000000000005</v>
+      </c>
+      <c r="F50">
         <f t="shared" si="37"/>
-        <v>51.370000000000005</v>
-      </c>
-      <c r="F50">
+        <v>12.5</v>
+      </c>
+      <c r="G50">
         <f t="shared" si="38"/>
-        <v>12.5</v>
-      </c>
-      <c r="G50">
-        <f t="shared" si="36"/>
         <v>57.370000000000005</v>
       </c>
       <c r="H50">
@@ -10674,15 +10674,15 @@
         <v>29</v>
       </c>
       <c r="E51">
+        <f t="shared" si="36"/>
+        <v>66.690000000000012</v>
+      </c>
+      <c r="F51">
         <f t="shared" si="37"/>
-        <v>66.690000000000012</v>
-      </c>
-      <c r="F51">
+        <v>15</v>
+      </c>
+      <c r="G51">
         <f t="shared" si="38"/>
-        <v>15</v>
-      </c>
-      <c r="G51">
-        <f t="shared" si="36"/>
         <v>70.190000000000012</v>
       </c>
       <c r="H51">
@@ -10707,15 +10707,15 @@
         <v>31</v>
       </c>
       <c r="E52">
+        <f t="shared" si="36"/>
+        <v>73.54000000000002</v>
+      </c>
+      <c r="F52">
         <f t="shared" si="37"/>
-        <v>73.54000000000002</v>
-      </c>
-      <c r="F52">
+        <v>17.5</v>
+      </c>
+      <c r="G52">
         <f t="shared" si="38"/>
-        <v>17.5</v>
-      </c>
-      <c r="G52">
-        <f t="shared" si="36"/>
         <v>74.54000000000002</v>
       </c>
       <c r="H52">
@@ -10740,15 +10740,15 @@
         <v>33</v>
       </c>
       <c r="E53">
+        <f t="shared" si="36"/>
+        <v>77.440000000000026</v>
+      </c>
+      <c r="F53">
         <f t="shared" si="37"/>
-        <v>77.440000000000026</v>
-      </c>
-      <c r="F53">
+        <v>20</v>
+      </c>
+      <c r="G53">
         <f t="shared" si="38"/>
-        <v>20</v>
-      </c>
-      <c r="G53">
-        <f t="shared" si="36"/>
         <v>75.940000000000012</v>
       </c>
       <c r="H53">
@@ -10773,15 +10773,15 @@
         <v>35</v>
       </c>
       <c r="E54">
+        <f t="shared" si="36"/>
+        <v>79.750000000000028</v>
+      </c>
+      <c r="F54">
         <f t="shared" si="37"/>
-        <v>79.750000000000028</v>
-      </c>
-      <c r="F54">
+        <v>22.5</v>
+      </c>
+      <c r="G54">
         <f t="shared" si="38"/>
-        <v>22.5</v>
-      </c>
-      <c r="G54">
-        <f t="shared" si="36"/>
         <v>75.750000000000014</v>
       </c>
       <c r="H54">
@@ -10806,15 +10806,15 @@
         <v>36</v>
       </c>
       <c r="E55">
+        <f t="shared" si="36"/>
+        <v>81.210000000000022</v>
+      </c>
+      <c r="F55">
         <f t="shared" si="37"/>
-        <v>81.210000000000022</v>
-      </c>
-      <c r="F55">
+        <v>25</v>
+      </c>
+      <c r="G55">
         <f t="shared" si="38"/>
-        <v>25</v>
-      </c>
-      <c r="G55">
-        <f t="shared" si="36"/>
         <v>74.710000000000008</v>
       </c>
       <c r="H55">
@@ -10839,15 +10839,15 @@
         <v>37</v>
       </c>
       <c r="E56">
+        <f t="shared" si="36"/>
+        <v>82.310000000000016</v>
+      </c>
+      <c r="F56">
         <f t="shared" si="37"/>
-        <v>82.310000000000016</v>
-      </c>
-      <c r="F56">
+        <v>27.5</v>
+      </c>
+      <c r="G56">
         <f t="shared" si="38"/>
-        <v>27.5</v>
-      </c>
-      <c r="G56">
-        <f t="shared" si="36"/>
         <v>73.310000000000016</v>
       </c>
       <c r="H56">
@@ -10872,15 +10872,15 @@
         <v>38</v>
       </c>
       <c r="E57">
+        <f t="shared" si="36"/>
+        <v>83.660000000000011</v>
+      </c>
+      <c r="F57">
         <f t="shared" si="37"/>
-        <v>83.660000000000011</v>
-      </c>
-      <c r="F57">
+        <v>30</v>
+      </c>
+      <c r="G57">
         <f t="shared" si="38"/>
-        <v>30</v>
-      </c>
-      <c r="G57">
-        <f t="shared" si="36"/>
         <v>72.160000000000025</v>
       </c>
       <c r="H57" s="11">
@@ -14866,6 +14866,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>